<commit_message>
Windows helper: one-click open in Power BI Desktop
</commit_message>
<xml_diff>
--- a/Functionality_Mapping_Table (1).xlsx
+++ b/Functionality_Mapping_Table (1).xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:N40"/>
+  <dimension ref="A1:M30"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -459,7 +459,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="26.4" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -2111,12 +2110,12 @@
       </c>
       <c r="H29" s="7" t="inlineStr">
         <is>
-          <t>'Open in Power BI' downloads a Power BI project (.pbip) with the data and a chart configured. Built behind an adapter interface so Tableau could be added.</t>
+          <t>'Open in Power BI' makes a Power BI project (.pbip) with the data and a chart configured through explicit model measures. On Windows, a one-time helper registers a locallens:// link so one click downloads the project and opens it in Power BI Desktop; elsewhere the project downloads. Built behind an adapter interface so Tableau could be added.</t>
         </is>
       </c>
       <c r="I29" s="7" t="inlineStr">
         <is>
-          <t>viz/adapters.py; viz/export_pbi.py</t>
+          <t>viz/adapters.py; viz/export_pbi.py; server/helper.py; server/links.py</t>
         </is>
       </c>
       <c r="J29" s="7" t="inlineStr">
@@ -2131,12 +2130,12 @@
       </c>
       <c r="L29" s="7" t="inlineStr">
         <is>
-          <t>tests/test_export_pbi.py (13); scripts/validate_pbip.py (Microsoft schema check)</t>
+          <t>tests/test_export_pbi.py (15); tests/test_helper.py (9); scripts/validate_pbip.py (Microsoft schema check)</t>
         </is>
       </c>
       <c r="M29" s="7" t="inlineStr">
         <is>
-          <t>NOT yet opened in Power BI Desktop (needs the Windows laptop). A file export, not a live API call. No Tableau.</t>
+          <t>NOT yet opened in Power BI Desktop and the helper is untested on Windows (needs the Windows laptop). A first version drew no chart because implicit measures were off; fixed with explicit measures, unconfirmed. Still a file export, not a live API call. No Tableau.</t>
         </is>
       </c>
     </row>
@@ -2205,16 +2204,6 @@
         </is>
       </c>
     </row>
-    <row r="31"/>
-    <row r="32"/>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
-    <row r="40"/>
   </sheetData>
   <autoFilter ref="A4:F29"/>
   <dataValidations count="2">

</xml_diff>

<commit_message>
Fine-tuned model: results, report, docs and mapping table
</commit_message>
<xml_diff>
--- a/Functionality_Mapping_Table (1).xlsx
+++ b/Functionality_Mapping_Table (1).xlsx
@@ -1277,17 +1277,17 @@
       </c>
       <c r="H16" s="7" t="inlineStr">
         <is>
-          <t>Domain-adapted via locally stored embeddings and a semantic layer: custom metrics, calculated columns, business rules, descriptions, and verified examples shown to the model. Embeddings match unfamiliar words by meaning.</t>
+          <t>Domain-adapted two ways. (1) Locally stored embeddings and a semantic layer: custom metrics, calculated columns, business rules, descriptions, verified examples. (2) A LoRA fine-tuned model (Qwen2.5-0.5B, trained on our own synthetic retail data) that fills the query frame: its own answer is right 95% of the time against 38% for the original model. The fine-tuned model is opt-in until one failure on a differently shaped dataset is fixed.</t>
         </is>
       </c>
       <c r="I16" s="7" t="inlineStr">
         <is>
-          <t>nlu/embeddings.py; data/semantic.py; data/registry.py</t>
+          <t>nlu/embeddings.py; data/semantic.py; data/registry.py; nlu/slm.py (shared prompt builder); finetune/ (data, training, export)</t>
         </is>
       </c>
       <c r="J16" s="7" t="inlineStr">
         <is>
-          <t>bge-small-en-v1.5 (Q8 GGUF), sqlglot-checked formulas</t>
+          <t>bge-small-en-v1.5 (Q8 GGUF); LoRA on Qwen2.5-0.5B-Instruct (Colab T4), GGUF Q8_0 / Q4_K_M; llama-cpp-python; sqlglot-checked formulas</t>
         </is>
       </c>
       <c r="K16" s="7" t="inlineStr">
@@ -1297,12 +1297,12 @@
       </c>
       <c r="L16" s="7" t="inlineStr">
         <is>
-          <t>tests/test_embeddings.py; tests/test_semantic.py; docs/EVAL.md (73% to 83% on held-out set 3)</t>
+          <t>docs/FINETUNING.md; eval/heldout4.py (frozen, tag heldout4-locked); docs/results/*; tests/test_finetune_data.py, test_prompt.py, test_embeddings.py</t>
         </is>
       </c>
       <c r="M16" s="7" t="inlineStr">
         <is>
-          <t>Fine-tuning the model itself (described embodiment, not in claim 7) is deliberately not done.</t>
+          <t>Held-out 4: final answers 82.4% to 85.8% with the rules on (0 lost, 8 gained, p = 0.008) and 50.2% to 83.7% with the model alone. Known failure: on a dataset where a question names two metrics (Wholesale customers) the fine-tuned model scores 13.7% against 86.3% for the original; fix planned (round 2).</t>
         </is>
       </c>
     </row>

</xml_diff>